<commit_message>
Week 2 README: walk through all 24 disagreements; correct consensus counts
</commit_message>
<xml_diff>
--- a/week-02/results/week2_evaluation_results.xlsx
+++ b/week-02/results/week2_evaluation_results.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="354">
   <si>
     <t xml:space="preserve">Resale Stack — Week 2 evaluation results</t>
   </si>
@@ -334,7 +334,7 @@
     <t xml:space="preserve">Models split among themselves</t>
   </si>
   <si>
-    <t xml:space="preserve">When three models converged against me, I was wrong most of the time. When they disagreed among themselves, I never was. (Counts reflect final causes; at first pass it was 8 of 17.)</t>
+    <t xml:space="preserve">Counted directly from disagreements_v2.csv (final causes). Consensus rows were label errors 59% of the time vs 43% for split rows: a modest hint on 24 rows, not a strong signal. An earlier version reported 13 of 17 and 0 of 7 in error.</t>
   </si>
   <si>
     <t xml:space="preserve">Clusters found</t>
@@ -889,13 +889,22 @@
     <t xml:space="preserve">Remaining disagreement was mostly me and my spec.</t>
   </si>
   <si>
-    <t xml:space="preserve">Model consensus flags my label errors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 of 17 consensus rows were label errors; 0 of 7 split rows.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use agreement among models to choose which labels to re-check.</t>
+    <t xml:space="preserve">Model consensus is only a modest hint of label error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 of 17 consensus rows were label errors vs 3 of 7 split rows (59% vs 43%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Too few rows to rely on. Re-check every disagreement, not just consensus ones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Six of 24 hinged on the title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L034, L065, L068, L070, L071 ("w/ Tags") and L123 ("Excellent Condition") put the deciding fact in the title, which I under-read.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read titles as evidence; check the labeling instructions say so.</t>
   </si>
   <si>
     <t xml:space="preserve">Correcting labels added 8–17 points</t>
@@ -3346,53 +3355,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B7" s="36" t="n">
         <v>12</v>
@@ -3419,7 +3428,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>4</v>
@@ -3446,7 +3455,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>0</v>
@@ -3473,7 +3482,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>0</v>
@@ -3500,7 +3509,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>0</v>
@@ -3527,7 +3536,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>2</v>
@@ -3554,7 +3563,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B13" s="35" t="n">
         <f aca="false">SUM(B7:B12)</f>
@@ -3587,7 +3596,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B14" s="37" t="str">
         <f aca="false">IF(H13=150,"OK","CHECK")</f>
@@ -3596,38 +3605,38 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B18" s="36" t="n">
         <v>15</v>
@@ -3654,7 +3663,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>8</v>
@@ -3681,7 +3690,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>0</v>
@@ -3708,7 +3717,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>0</v>
@@ -3735,7 +3744,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>0</v>
@@ -3762,7 +3771,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>0</v>
@@ -3789,7 +3798,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B24" s="35" t="n">
         <f aca="false">SUM(B18:B23)</f>
@@ -3822,7 +3831,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B25" s="37" t="str">
         <f aca="false">IF(H24=150,"OK","CHECK")</f>
@@ -3831,38 +3840,38 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B29" s="36" t="n">
         <v>16</v>
@@ -3889,7 +3898,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B30" s="9" t="n">
         <v>0</v>
@@ -3916,7 +3925,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B31" s="9" t="n">
         <v>0</v>
@@ -3943,7 +3952,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B32" s="9" t="n">
         <v>0</v>
@@ -3970,7 +3979,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B33" s="9" t="n">
         <v>0</v>
@@ -3997,7 +4006,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B34" s="9" t="n">
         <v>0</v>
@@ -4024,7 +4033,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B35" s="35" t="n">
         <f aca="false">SUM(B29:B34)</f>
@@ -4057,7 +4066,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B36" s="37" t="str">
         <f aca="false">IF(H35=150,"OK","CHECK")</f>
@@ -4089,53 +4098,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B7" s="36" t="n">
         <v>14</v>
@@ -4162,7 +4171,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>5</v>
@@ -4189,7 +4198,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>0</v>
@@ -4216,7 +4225,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>0</v>
@@ -4243,7 +4252,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>0</v>
@@ -4270,7 +4279,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>1</v>
@@ -4297,7 +4306,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B13" s="35" t="n">
         <f aca="false">SUM(B7:B12)</f>
@@ -4330,7 +4339,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B14" s="37" t="str">
         <f aca="false">IF(H13=150,"OK","CHECK")</f>
@@ -4339,38 +4348,38 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B18" s="36" t="n">
         <v>14</v>
@@ -4397,7 +4406,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>6</v>
@@ -4424,7 +4433,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>0</v>
@@ -4451,7 +4460,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>0</v>
@@ -4478,7 +4487,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>0</v>
@@ -4505,7 +4514,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>3</v>
@@ -4532,7 +4541,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B24" s="35" t="n">
         <f aca="false">SUM(B18:B23)</f>
@@ -4565,7 +4574,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B25" s="37" t="str">
         <f aca="false">IF(H24=150,"OK","CHECK")</f>
@@ -4574,38 +4583,38 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B29" s="36" t="n">
         <v>15</v>
@@ -4632,7 +4641,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B30" s="9" t="n">
         <v>0</v>
@@ -4659,7 +4668,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B31" s="9" t="n">
         <v>0</v>
@@ -4686,7 +4695,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B32" s="9" t="n">
         <v>0</v>
@@ -4713,7 +4722,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B33" s="9" t="n">
         <v>0</v>
@@ -4740,7 +4749,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B34" s="9" t="n">
         <v>0</v>
@@ -4767,7 +4776,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B35" s="35" t="n">
         <f aca="false">SUM(B29:B34)</f>
@@ -4800,7 +4809,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B36" s="37" t="str">
         <f aca="false">IF(H35=150,"OK","CHECK")</f>
@@ -4832,43 +4841,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B6" s="36" t="n">
         <v>2</v>
@@ -4895,7 +4904,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>5</v>
@@ -4922,7 +4931,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>0</v>
@@ -4949,7 +4958,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>0</v>
@@ -4976,7 +4985,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>0</v>
@@ -5003,7 +5012,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>0</v>
@@ -5030,7 +5039,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B12" s="35" t="n">
         <f aca="false">SUM(B6:B11)</f>
@@ -5063,7 +5072,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B13" s="37" t="str">
         <f aca="false">IF(H12=37,"OK","CHECK")</f>
@@ -5072,38 +5081,38 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B17" s="36" t="n">
         <v>3</v>
@@ -5130,7 +5139,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B18" s="9" t="n">
         <v>4</v>
@@ -5157,7 +5166,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>0</v>
@@ -5184,7 +5193,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>0</v>
@@ -5211,7 +5220,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>0</v>
@@ -5238,7 +5247,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>0</v>
@@ -5265,7 +5274,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B23" s="35" t="n">
         <f aca="false">SUM(B17:B22)</f>
@@ -5298,7 +5307,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B24" s="37" t="str">
         <f aca="false">IF(H23=37,"OK","CHECK")</f>
@@ -5307,38 +5316,38 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B28" s="36" t="n">
         <v>2</v>
@@ -5365,7 +5374,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B29" s="9" t="n">
         <v>1</v>
@@ -5392,7 +5401,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B30" s="9" t="n">
         <v>0</v>
@@ -5419,7 +5428,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B31" s="9" t="n">
         <v>0</v>
@@ -5446,7 +5455,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B32" s="9" t="n">
         <v>0</v>
@@ -5473,7 +5482,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B33" s="9" t="n">
         <v>0</v>
@@ -5500,7 +5509,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B34" s="35" t="n">
         <f aca="false">SUM(B28:B33)</f>
@@ -5533,7 +5542,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B35" s="37" t="str">
         <f aca="false">IF(H34=37,"OK","CHECK")</f>
@@ -5564,26 +5573,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B4" s="38" t="n">
         <v>8</v>
@@ -5598,7 +5607,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B5" s="38" t="n">
         <v>8</v>
@@ -5613,7 +5622,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -5795,11 +5804,11 @@
         <v>17</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D14" s="29" t="n">
         <f aca="false">C14/B14</f>
-        <v>0.764705882352941</v>
+        <v>0.588235294117647</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5810,11 +5819,11 @@
         <v>7</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D15" s="29" t="n">
         <f aca="false">C15/B15</f>
-        <v>0</v>
+        <v>0.428571428571429</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6825,7 +6834,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -7004,6 +7013,20 @@
       </c>
       <c r="D14" s="33" t="s">
         <v>293</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="32" t="s">
+        <v>294</v>
+      </c>
+      <c r="C15" s="33" t="s">
+        <v>295</v>
+      </c>
+      <c r="D15" s="33" t="s">
+        <v>296</v>
       </c>
     </row>
   </sheetData>
@@ -7031,103 +7054,103 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="35" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="35" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="35" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="35" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="35" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="35" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="35" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="35" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="35" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="35" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="35" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
   </sheetData>
@@ -7155,48 +7178,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B7" s="36" t="n">
         <v>8</v>
@@ -7223,7 +7246,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>8</v>
@@ -7250,7 +7273,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>0</v>
@@ -7277,7 +7300,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>0</v>
@@ -7304,7 +7327,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>0</v>
@@ -7331,7 +7354,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>2</v>
@@ -7358,7 +7381,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B13" s="35" t="n">
         <f aca="false">SUM(B7:B12)</f>
@@ -7391,7 +7414,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B14" s="37" t="str">
         <f aca="false">IF(H13=150,"OK","CHECK")</f>
@@ -7400,38 +7423,38 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B18" s="36" t="n">
         <v>9</v>
@@ -7458,7 +7481,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>9</v>
@@ -7485,7 +7508,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>0</v>
@@ -7512,7 +7535,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>0</v>
@@ -7539,7 +7562,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>0</v>
@@ -7566,7 +7589,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>5</v>
@@ -7593,7 +7616,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B24" s="35" t="n">
         <f aca="false">SUM(B18:B23)</f>
@@ -7626,7 +7649,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B25" s="37" t="str">
         <f aca="false">IF(H24=150,"OK","CHECK")</f>
@@ -7635,38 +7658,38 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B29" s="36" t="n">
         <v>9</v>
@@ -7693,7 +7716,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B30" s="9" t="n">
         <v>4</v>
@@ -7720,7 +7743,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B31" s="9" t="n">
         <v>0</v>
@@ -7747,7 +7770,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B32" s="9" t="n">
         <v>0</v>
@@ -7774,7 +7797,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B33" s="9" t="n">
         <v>0</v>
@@ -7801,7 +7824,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B34" s="9" t="n">
         <v>3</v>
@@ -7828,7 +7851,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B35" s="35" t="n">
         <f aca="false">SUM(B29:B34)</f>
@@ -7861,7 +7884,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B36" s="37" t="str">
         <f aca="false">IF(H35=150,"OK","CHECK")</f>
@@ -7893,48 +7916,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B7" s="36" t="n">
         <v>9</v>
@@ -7961,7 +7984,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>10</v>
@@ -7988,7 +8011,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>0</v>
@@ -8015,7 +8038,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>0</v>
@@ -8042,7 +8065,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>0</v>
@@ -8069,7 +8092,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>1</v>
@@ -8096,7 +8119,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B13" s="35" t="n">
         <f aca="false">SUM(B7:B12)</f>
@@ -8129,7 +8152,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B14" s="37" t="str">
         <f aca="false">IF(H13=150,"OK","CHECK")</f>
@@ -8138,38 +8161,38 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B18" s="36" t="n">
         <v>10</v>
@@ -8196,7 +8219,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>7</v>
@@ -8223,7 +8246,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>0</v>
@@ -8250,7 +8273,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>0</v>
@@ -8277,7 +8300,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>0</v>
@@ -8304,7 +8327,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>6</v>
@@ -8331,7 +8354,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B24" s="35" t="n">
         <f aca="false">SUM(B18:B23)</f>
@@ -8364,7 +8387,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B25" s="37" t="str">
         <f aca="false">IF(H24=150,"OK","CHECK")</f>
@@ -8373,38 +8396,38 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B29" s="36" t="n">
         <v>9</v>
@@ -8431,7 +8454,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B30" s="9" t="n">
         <v>3</v>
@@ -8458,7 +8481,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B31" s="9" t="n">
         <v>0</v>
@@ -8485,7 +8508,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B32" s="9" t="n">
         <v>0</v>
@@ -8512,7 +8535,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B33" s="9" t="n">
         <v>0</v>
@@ -8539,7 +8562,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B34" s="9" t="n">
         <v>3</v>
@@ -8566,7 +8589,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B35" s="35" t="n">
         <f aca="false">SUM(B29:B34)</f>
@@ -8599,7 +8622,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B36" s="37" t="str">
         <f aca="false">IF(H35=150,"OK","CHECK")</f>

</xml_diff>